<commit_message>
Uploading the PCB files kanboard #7406
</commit_message>
<xml_diff>
--- a/Documents/HardwareCheckList_V43 3 1.xlsx
+++ b/Documents/HardwareCheckList_V43 3 1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Documents\Qx_HW_CheckList\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspace\KiCad\Project_2\Documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FE94BB9-7AD4-48E0-8D76-5A08E74853F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9CE1C1B-0DE3-46EC-831A-D0E38B177B4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="1" xr2:uid="{68843EE4-1B9F-4521-A53B-766934041111}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" firstSheet="1" activeTab="2" xr2:uid="{68843EE4-1B9F-4521-A53B-766934041111}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Requirments" sheetId="5" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="584" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="585" uniqueCount="266">
   <si>
     <t>QUANTTRONIX HARDWARE CHECKLIST</t>
   </si>
@@ -856,6 +856,9 @@
   </si>
   <si>
     <t>7ot parallel w wahed tany in series</t>
+  </si>
+  <si>
+    <t>Applied 3la el I2C</t>
   </si>
 </sst>
 </file>
@@ -1302,54 +1305,6 @@
     <xf numFmtId="0" fontId="6" fillId="11" borderId="1" xfId="10" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -1368,6 +1323,54 @@
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="1" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" xfId="5" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="8" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="1" xfId="10" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="1" xfId="9" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="0" xfId="6" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="11">
@@ -1855,19 +1858,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="31.5" x14ac:dyDescent="0.5">
-      <c r="A1" s="81" t="s">
+      <c r="A1" s="88" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="81"/>
+      <c r="B1" s="88"/>
       <c r="C1" s="3"/>
       <c r="D1" s="5"/>
       <c r="E1" s="5"/>
     </row>
     <row r="2" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
-      <c r="A2" s="82" t="s">
+      <c r="A2" s="89" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="82"/>
+      <c r="B2" s="89"/>
       <c r="C2" s="4"/>
     </row>
     <row r="3" spans="1:5" ht="23.25" x14ac:dyDescent="0.25">
@@ -1902,32 +1905,32 @@
     <col min="4" max="4" width="164" style="6" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="21.85546875" style="54" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="20.28515625" style="56" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="101.7109375" style="96" customWidth="1"/>
+    <col min="7" max="7" width="101.7109375" style="80" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="33.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="78" t="s">
+      <c r="A1" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="78"/>
-      <c r="C1" s="78"/>
-      <c r="D1" s="78"/>
-      <c r="E1" s="78"/>
-      <c r="F1" s="78"/>
-      <c r="G1" s="78"/>
+      <c r="B1" s="85"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="E1" s="85"/>
+      <c r="F1" s="85"/>
+      <c r="G1" s="85"/>
       <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="79" t="s">
+      <c r="A2" s="86" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="79"/>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="79"/>
-      <c r="G2" s="79"/>
+      <c r="B2" s="86"/>
+      <c r="C2" s="86"/>
+      <c r="D2" s="86"/>
+      <c r="E2" s="86"/>
+      <c r="F2" s="86"/>
+      <c r="G2" s="86"/>
       <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" s="13" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
@@ -1947,7 +1950,7 @@
       <c r="H3" s="15"/>
     </row>
     <row r="4" spans="1:8" s="13" customFormat="1" ht="23.25" x14ac:dyDescent="0.35">
-      <c r="A4" s="76" t="s">
+      <c r="A4" s="83" t="s">
         <v>7</v>
       </c>
       <c r="B4" s="41">
@@ -1963,15 +1966,15 @@
         <v>10</v>
       </c>
       <c r="F4" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="97" t="s">
+        <v>223</v>
+      </c>
+      <c r="G4" s="81" t="s">
         <v>225</v>
       </c>
       <c r="H4" s="15"/>
     </row>
     <row r="5" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="76"/>
+      <c r="A5" s="83"/>
       <c r="B5" s="41">
         <v>2</v>
       </c>
@@ -1983,13 +1986,13 @@
         <v>10</v>
       </c>
       <c r="F5" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G5" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G5" s="75"/>
       <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="76"/>
+      <c r="A6" s="83"/>
       <c r="B6" s="41">
         <v>3</v>
       </c>
@@ -2001,14 +2004,14 @@
         <v>10</v>
       </c>
       <c r="F6" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G6" s="92" t="s">
+        <v>223</v>
+      </c>
+      <c r="G6" s="76" t="s">
         <v>226</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" s="76"/>
+      <c r="A7" s="83"/>
       <c r="B7" s="41">
         <v>4</v>
       </c>
@@ -2020,15 +2023,15 @@
         <v>10</v>
       </c>
       <c r="F7" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G7" s="75" t="s">
         <v>227</v>
       </c>
       <c r="H7" s="8"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A8" s="76"/>
+      <c r="A8" s="83"/>
       <c r="B8" s="41">
         <v>5</v>
       </c>
@@ -2040,15 +2043,15 @@
         <v>10</v>
       </c>
       <c r="F8" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G8" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G8" s="75" t="s">
         <v>228</v>
       </c>
       <c r="H8" s="8"/>
     </row>
     <row r="9" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A9" s="76"/>
+      <c r="A9" s="83"/>
       <c r="B9" s="41">
         <v>6</v>
       </c>
@@ -2058,15 +2061,15 @@
       </c>
       <c r="E9" s="50"/>
       <c r="F9" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G9" s="75" t="s">
         <v>229</v>
       </c>
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A10" s="76"/>
+      <c r="A10" s="83"/>
       <c r="B10" s="41">
         <v>7</v>
       </c>
@@ -2078,15 +2081,15 @@
         <v>10</v>
       </c>
       <c r="F10" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G10" s="75" t="s">
         <v>230</v>
       </c>
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A11" s="76"/>
+      <c r="A11" s="83"/>
       <c r="B11" s="41">
         <v>8</v>
       </c>
@@ -2098,15 +2101,15 @@
         <v>10</v>
       </c>
       <c r="F11" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G11" s="75" t="s">
         <v>231</v>
       </c>
       <c r="H11" s="8"/>
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A12" s="76"/>
+      <c r="A12" s="83"/>
       <c r="B12" s="41">
         <v>9</v>
       </c>
@@ -2118,15 +2121,15 @@
         <v>10</v>
       </c>
       <c r="F12" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G12" s="93" t="s">
+        <v>223</v>
+      </c>
+      <c r="G12" s="77" t="s">
         <v>232</v>
       </c>
       <c r="H12" s="8"/>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A13" s="76"/>
+      <c r="A13" s="83"/>
       <c r="B13" s="41">
         <v>10</v>
       </c>
@@ -2138,15 +2141,15 @@
         <v>10</v>
       </c>
       <c r="F13" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G13" s="75" t="s">
         <v>233</v>
       </c>
       <c r="H13" s="8"/>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A14" s="76"/>
+      <c r="A14" s="83"/>
       <c r="B14" s="41">
         <v>11</v>
       </c>
@@ -2158,15 +2161,15 @@
         <v>10</v>
       </c>
       <c r="F14" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G14" s="75" t="s">
         <v>233</v>
       </c>
       <c r="H14" s="8"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A15" s="76"/>
+      <c r="A15" s="83"/>
       <c r="B15" s="41">
         <v>12</v>
       </c>
@@ -2178,15 +2181,15 @@
         <v>10</v>
       </c>
       <c r="F15" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G15" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G15" s="75" t="s">
         <v>234</v>
       </c>
       <c r="H15" s="8"/>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A16" s="76"/>
+      <c r="A16" s="83"/>
       <c r="B16" s="41">
         <v>13</v>
       </c>
@@ -2198,15 +2201,15 @@
         <v>10</v>
       </c>
       <c r="F16" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G16" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G16" s="75" t="s">
         <v>235</v>
       </c>
       <c r="H16" s="8"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="76"/>
+      <c r="A17" s="83"/>
       <c r="B17" s="41">
         <v>14</v>
       </c>
@@ -2218,14 +2221,14 @@
         <v>10</v>
       </c>
       <c r="F17" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G17" s="92" t="s">
+        <v>223</v>
+      </c>
+      <c r="G17" s="76" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A18" s="76"/>
+      <c r="A18" s="83"/>
       <c r="B18" s="41">
         <v>15</v>
       </c>
@@ -2237,15 +2240,15 @@
         <v>10</v>
       </c>
       <c r="F18" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G18" s="93" t="s">
+        <v>223</v>
+      </c>
+      <c r="G18" s="77" t="s">
         <v>237</v>
       </c>
       <c r="H18" s="8"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A19" s="76"/>
+      <c r="A19" s="83"/>
       <c r="B19" s="41">
         <v>16</v>
       </c>
@@ -2257,15 +2260,15 @@
         <v>10</v>
       </c>
       <c r="F19" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G19" s="93" t="s">
+        <v>222</v>
+      </c>
+      <c r="G19" s="77" t="s">
         <v>238</v>
       </c>
       <c r="H19" s="8"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A20" s="76"/>
+      <c r="A20" s="83"/>
       <c r="B20" s="41">
         <v>17</v>
       </c>
@@ -2277,15 +2280,15 @@
         <v>10</v>
       </c>
       <c r="F20" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G20" s="93" t="s">
+        <v>222</v>
+      </c>
+      <c r="G20" s="77" t="s">
         <v>239</v>
       </c>
       <c r="H20" s="8"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A21" s="77" t="s">
+      <c r="A21" s="84" t="s">
         <v>28</v>
       </c>
       <c r="B21" s="42">
@@ -2299,14 +2302,14 @@
         <v>10</v>
       </c>
       <c r="F21" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G21" s="92" t="s">
+        <v>223</v>
+      </c>
+      <c r="G21" s="76" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A22" s="77"/>
+      <c r="A22" s="84"/>
       <c r="B22" s="42">
         <v>19</v>
       </c>
@@ -2318,15 +2321,15 @@
         <v>31</v>
       </c>
       <c r="F22" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G22" s="91">
+        <v>223</v>
+      </c>
+      <c r="G22" s="75">
         <v>2.54</v>
       </c>
       <c r="H22" s="8"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A23" s="77"/>
+      <c r="A23" s="84"/>
       <c r="B23" s="42">
         <v>20</v>
       </c>
@@ -2338,15 +2341,15 @@
         <v>10</v>
       </c>
       <c r="F23" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G23" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G23" s="75" t="s">
         <v>241</v>
       </c>
       <c r="H23" s="8"/>
     </row>
     <row r="24" spans="1:8" ht="37.5" x14ac:dyDescent="0.3">
-      <c r="A24" s="77"/>
+      <c r="A24" s="84"/>
       <c r="B24" s="42">
         <v>21</v>
       </c>
@@ -2358,15 +2361,15 @@
         <v>10</v>
       </c>
       <c r="F24" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G24" s="96" t="s">
+        <v>223</v>
+      </c>
+      <c r="G24" s="80" t="s">
         <v>243</v>
       </c>
       <c r="H24" s="8"/>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A25" s="77"/>
+      <c r="A25" s="84"/>
       <c r="B25" s="42">
         <v>22</v>
       </c>
@@ -2378,14 +2381,14 @@
         <v>10</v>
       </c>
       <c r="F25" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G25" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G25" s="75" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A26" s="77"/>
+      <c r="A26" s="84"/>
       <c r="B26" s="42">
         <v>23</v>
       </c>
@@ -2397,15 +2400,15 @@
         <v>10</v>
       </c>
       <c r="F26" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G26" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G26" s="75" t="s">
         <v>244</v>
       </c>
       <c r="H26" s="8"/>
     </row>
     <row r="27" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="77"/>
+      <c r="A27" s="84"/>
       <c r="B27" s="42">
         <v>24</v>
       </c>
@@ -2417,13 +2420,15 @@
         <v>10</v>
       </c>
       <c r="F27" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G27" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G27" s="75" t="s">
+        <v>265</v>
+      </c>
       <c r="H27" s="8"/>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A28" s="77"/>
+      <c r="A28" s="84"/>
       <c r="B28" s="42">
         <v>25</v>
       </c>
@@ -2435,15 +2440,15 @@
         <v>38</v>
       </c>
       <c r="F28" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G28" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G28" s="75" t="s">
         <v>245</v>
       </c>
       <c r="H28" s="8"/>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A29" s="77"/>
+      <c r="A29" s="84"/>
       <c r="B29" s="42">
         <v>26</v>
       </c>
@@ -2455,15 +2460,15 @@
         <v>38</v>
       </c>
       <c r="F29" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G29" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G29" s="75" t="s">
         <v>246</v>
       </c>
       <c r="H29" s="8"/>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A30" s="77"/>
+      <c r="A30" s="84"/>
       <c r="B30" s="42">
         <v>27</v>
       </c>
@@ -2475,15 +2480,15 @@
         <v>38</v>
       </c>
       <c r="F30" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G30" s="96" t="s">
+        <v>222</v>
+      </c>
+      <c r="G30" s="80" t="s">
         <v>247</v>
       </c>
       <c r="H30" s="8"/>
     </row>
     <row r="31" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A31" s="77"/>
+      <c r="A31" s="84"/>
       <c r="B31" s="42">
         <v>28</v>
       </c>
@@ -2495,15 +2500,15 @@
         <v>38</v>
       </c>
       <c r="F31" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G31" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G31" s="75" t="s">
         <v>248</v>
       </c>
       <c r="H31" s="8"/>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A32" s="77"/>
+      <c r="A32" s="84"/>
       <c r="B32" s="42">
         <v>29</v>
       </c>
@@ -2515,15 +2520,15 @@
         <v>38</v>
       </c>
       <c r="F32" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G32" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G32" s="75" t="s">
         <v>249</v>
       </c>
       <c r="H32" s="8"/>
     </row>
     <row r="33" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A33" s="77"/>
+      <c r="A33" s="84"/>
       <c r="B33" s="42">
         <v>30</v>
       </c>
@@ -2535,15 +2540,15 @@
         <v>38</v>
       </c>
       <c r="F33" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G33" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G33" s="75" t="s">
         <v>251</v>
       </c>
       <c r="H33" s="8"/>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A34" s="77"/>
+      <c r="A34" s="84"/>
       <c r="B34" s="42">
         <v>31</v>
       </c>
@@ -2555,15 +2560,15 @@
         <v>38</v>
       </c>
       <c r="F34" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G34" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G34" s="75" t="s">
         <v>252</v>
       </c>
       <c r="H34" s="8"/>
     </row>
     <row r="35" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A35" s="77"/>
+      <c r="A35" s="84"/>
       <c r="B35" s="42">
         <v>32</v>
       </c>
@@ -2575,15 +2580,15 @@
         <v>38</v>
       </c>
       <c r="F35" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G35" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G35" s="75" t="s">
         <v>253</v>
       </c>
       <c r="H35" s="8"/>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A36" s="77"/>
+      <c r="A36" s="84"/>
       <c r="B36" s="42">
         <v>33</v>
       </c>
@@ -2595,13 +2600,13 @@
         <v>38</v>
       </c>
       <c r="F36" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G36" s="91"/>
+        <v>222</v>
+      </c>
+      <c r="G36" s="75"/>
       <c r="H36" s="8"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A37" s="77"/>
+      <c r="A37" s="84"/>
       <c r="B37" s="42">
         <v>34</v>
       </c>
@@ -2613,12 +2618,12 @@
         <v>38</v>
       </c>
       <c r="F37" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G37" s="92"/>
+        <v>222</v>
+      </c>
+      <c r="G37" s="76"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A38" s="77"/>
+      <c r="A38" s="84"/>
       <c r="B38" s="42">
         <v>35</v>
       </c>
@@ -2630,13 +2635,13 @@
         <v>38</v>
       </c>
       <c r="F38" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G38" s="91"/>
+        <v>222</v>
+      </c>
+      <c r="G38" s="75"/>
       <c r="H38" s="8"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A39" s="77"/>
+      <c r="A39" s="84"/>
       <c r="B39" s="42">
         <v>36</v>
       </c>
@@ -2648,14 +2653,14 @@
         <v>50</v>
       </c>
       <c r="F39" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G39" s="92" t="s">
+        <v>222</v>
+      </c>
+      <c r="G39" s="76" t="s">
         <v>250</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A40" s="77"/>
+      <c r="A40" s="84"/>
       <c r="B40" s="42">
         <v>37</v>
       </c>
@@ -2667,13 +2672,13 @@
         <v>10</v>
       </c>
       <c r="F40" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G40" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G40" s="75"/>
       <c r="H40" s="8"/>
     </row>
     <row r="41" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A41" s="77"/>
+      <c r="A41" s="84"/>
       <c r="B41" s="42">
         <v>38</v>
       </c>
@@ -2685,15 +2690,15 @@
         <v>10</v>
       </c>
       <c r="F41" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G41" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G41" s="75" t="s">
         <v>254</v>
       </c>
       <c r="H41" s="8"/>
     </row>
     <row r="42" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A42" s="77"/>
+      <c r="A42" s="84"/>
       <c r="B42" s="42">
         <v>39</v>
       </c>
@@ -2707,13 +2712,13 @@
       <c r="F42" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G42" s="91" t="s">
+      <c r="G42" s="75" t="s">
         <v>255</v>
       </c>
       <c r="H42" s="8"/>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A43" s="77"/>
+      <c r="A43" s="84"/>
       <c r="B43" s="42">
         <v>40</v>
       </c>
@@ -2725,13 +2730,13 @@
         <v>10</v>
       </c>
       <c r="F43" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G43" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G43" s="75"/>
       <c r="H43" s="8"/>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A44" s="77"/>
+      <c r="A44" s="84"/>
       <c r="B44" s="42">
         <v>41</v>
       </c>
@@ -2743,13 +2748,13 @@
         <v>10</v>
       </c>
       <c r="F44" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G44" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G44" s="75"/>
       <c r="H44" s="8"/>
     </row>
     <row r="45" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A45" s="77"/>
+      <c r="A45" s="84"/>
       <c r="B45" s="42">
         <v>42</v>
       </c>
@@ -2761,15 +2766,15 @@
         <v>10</v>
       </c>
       <c r="F45" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G45" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G45" s="75" t="s">
         <v>256</v>
       </c>
       <c r="H45" s="8"/>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A46" s="77"/>
+      <c r="A46" s="84"/>
       <c r="B46" s="42">
         <v>43</v>
       </c>
@@ -2783,13 +2788,13 @@
         <v>10</v>
       </c>
       <c r="F46" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G46" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G46" s="75"/>
       <c r="H46" s="8"/>
     </row>
     <row r="47" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A47" s="80" t="s">
+      <c r="A47" s="87" t="s">
         <v>58</v>
       </c>
       <c r="B47" s="43">
@@ -2803,15 +2808,15 @@
         <v>10</v>
       </c>
       <c r="F47" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G47" s="91"/>
+        <v>222</v>
+      </c>
+      <c r="G47" s="75"/>
       <c r="H47" s="8" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="48" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A48" s="80"/>
+      <c r="A48" s="87"/>
       <c r="B48" s="43">
         <v>45</v>
       </c>
@@ -2823,13 +2828,13 @@
         <v>10</v>
       </c>
       <c r="F48" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G48" s="91"/>
+        <v>222</v>
+      </c>
+      <c r="G48" s="75"/>
       <c r="H48" s="8"/>
     </row>
     <row r="49" spans="1:8" ht="56.25" x14ac:dyDescent="0.25">
-      <c r="A49" s="80"/>
+      <c r="A49" s="87"/>
       <c r="B49" s="43">
         <v>46</v>
       </c>
@@ -2841,15 +2846,15 @@
         <v>10</v>
       </c>
       <c r="F49" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G49" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G49" s="75" t="s">
         <v>257</v>
       </c>
       <c r="H49" s="8"/>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A50" s="80"/>
+      <c r="A50" s="87"/>
       <c r="B50" s="43">
         <v>47</v>
       </c>
@@ -2861,13 +2866,13 @@
         <v>10</v>
       </c>
       <c r="F50" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G50" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G50" s="75"/>
       <c r="H50" s="8"/>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A51" s="80"/>
+      <c r="A51" s="87"/>
       <c r="B51" s="43">
         <v>48</v>
       </c>
@@ -2879,12 +2884,12 @@
         <v>10</v>
       </c>
       <c r="F51" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G51" s="94"/>
+        <v>223</v>
+      </c>
+      <c r="G51" s="78"/>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A52" s="76" t="s">
+      <c r="A52" s="83" t="s">
         <v>65</v>
       </c>
       <c r="B52" s="41">
@@ -2902,11 +2907,11 @@
       <c r="F52" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G52" s="91"/>
+      <c r="G52" s="75"/>
       <c r="H52" s="8"/>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" s="76"/>
+      <c r="A53" s="83"/>
       <c r="B53" s="41">
         <v>50</v>
       </c>
@@ -2918,14 +2923,14 @@
         <v>10</v>
       </c>
       <c r="F53" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G53" s="92" t="s">
+        <v>223</v>
+      </c>
+      <c r="G53" s="76" t="s">
         <v>258</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A54" s="76"/>
+      <c r="A54" s="83"/>
       <c r="B54" s="41">
         <v>51</v>
       </c>
@@ -2937,13 +2942,13 @@
         <v>10</v>
       </c>
       <c r="F54" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G54" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G54" s="75"/>
       <c r="H54" s="8"/>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A55" s="76"/>
+      <c r="A55" s="83"/>
       <c r="B55" s="41">
         <v>52</v>
       </c>
@@ -2955,15 +2960,15 @@
         <v>10</v>
       </c>
       <c r="F55" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G55" s="91" t="s">
+        <v>224</v>
+      </c>
+      <c r="G55" s="75" t="s">
         <v>259</v>
       </c>
       <c r="H55" s="8"/>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A56" s="76"/>
+      <c r="A56" s="83"/>
       <c r="B56" s="41">
         <v>53</v>
       </c>
@@ -2975,13 +2980,13 @@
         <v>10</v>
       </c>
       <c r="F56" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G56" s="91"/>
+        <v>222</v>
+      </c>
+      <c r="G56" s="75"/>
       <c r="H56" s="8"/>
     </row>
     <row r="57" spans="1:8" ht="37.5" x14ac:dyDescent="0.25">
-      <c r="A57" s="76"/>
+      <c r="A57" s="83"/>
       <c r="B57" s="41">
         <v>54</v>
       </c>
@@ -2993,15 +2998,15 @@
         <v>10</v>
       </c>
       <c r="F57" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G57" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G57" s="75" t="s">
         <v>260</v>
       </c>
       <c r="H57" s="8"/>
     </row>
     <row r="58" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A58" s="76"/>
+      <c r="A58" s="83"/>
       <c r="B58" s="41">
         <v>55</v>
       </c>
@@ -3013,13 +3018,13 @@
         <v>10</v>
       </c>
       <c r="F58" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G58" s="91"/>
+        <v>224</v>
+      </c>
+      <c r="G58" s="75"/>
       <c r="H58" s="8"/>
     </row>
     <row r="59" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A59" s="76"/>
+      <c r="A59" s="83"/>
       <c r="B59" s="41">
         <v>56</v>
       </c>
@@ -3031,13 +3036,13 @@
         <v>10</v>
       </c>
       <c r="F59" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G59" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G59" s="75"/>
       <c r="H59" s="8"/>
     </row>
     <row r="60" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A60" s="76"/>
+      <c r="A60" s="83"/>
       <c r="B60" s="41">
         <v>57</v>
       </c>
@@ -3051,11 +3056,11 @@
       <c r="F60" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G60" s="91"/>
+      <c r="G60" s="75"/>
       <c r="H60" s="8"/>
     </row>
     <row r="61" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A61" s="76"/>
+      <c r="A61" s="83"/>
       <c r="B61" s="41">
         <v>58</v>
       </c>
@@ -3069,11 +3074,11 @@
       <c r="F61" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G61" s="91"/>
+      <c r="G61" s="75"/>
       <c r="H61" s="8"/>
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A62" s="76"/>
+      <c r="A62" s="83"/>
       <c r="B62" s="41">
         <v>59</v>
       </c>
@@ -3085,13 +3090,13 @@
         <v>261</v>
       </c>
       <c r="F62" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G62" s="91"/>
+        <v>222</v>
+      </c>
+      <c r="G62" s="75"/>
       <c r="H62" s="8"/>
     </row>
     <row r="63" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A63" s="77" t="s">
+      <c r="A63" s="84" t="s">
         <v>78</v>
       </c>
       <c r="B63" s="42">
@@ -3105,13 +3110,13 @@
         <v>10</v>
       </c>
       <c r="F63" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G63" s="91"/>
+        <v>222</v>
+      </c>
+      <c r="G63" s="75"/>
       <c r="H63" s="8"/>
     </row>
     <row r="64" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A64" s="77"/>
+      <c r="A64" s="84"/>
       <c r="B64" s="42">
         <v>61</v>
       </c>
@@ -3123,15 +3128,15 @@
         <v>10</v>
       </c>
       <c r="F64" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G64" s="91" t="s">
+        <v>223</v>
+      </c>
+      <c r="G64" s="75" t="s">
         <v>262</v>
       </c>
       <c r="H64" s="8"/>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A65" s="77"/>
+      <c r="A65" s="84"/>
       <c r="B65" s="42">
         <v>62</v>
       </c>
@@ -3143,13 +3148,13 @@
         <v>10</v>
       </c>
       <c r="F65" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G65" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G65" s="75"/>
       <c r="H65" s="8"/>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A66" s="77"/>
+      <c r="A66" s="84"/>
       <c r="B66" s="42">
         <v>63</v>
       </c>
@@ -3161,13 +3166,13 @@
         <v>10</v>
       </c>
       <c r="F66" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G66" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G66" s="75"/>
       <c r="H66" s="8"/>
     </row>
     <row r="67" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A67" s="77"/>
+      <c r="A67" s="84"/>
       <c r="B67" s="42">
         <v>64</v>
       </c>
@@ -3179,15 +3184,15 @@
         <v>10</v>
       </c>
       <c r="F67" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G67" s="91" t="s">
+        <v>222</v>
+      </c>
+      <c r="G67" s="75" t="s">
         <v>263</v>
       </c>
       <c r="H67" s="8"/>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A68" s="77"/>
+      <c r="A68" s="84"/>
       <c r="B68" s="42">
         <v>65</v>
       </c>
@@ -3201,11 +3206,11 @@
       <c r="F68" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G68" s="91"/>
+      <c r="G68" s="75"/>
       <c r="H68" s="8"/>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A69" s="77"/>
+      <c r="A69" s="84"/>
       <c r="B69" s="42">
         <v>66</v>
       </c>
@@ -3217,13 +3222,13 @@
         <v>10</v>
       </c>
       <c r="F69" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G69" s="91"/>
+        <v>224</v>
+      </c>
+      <c r="G69" s="75"/>
       <c r="H69" s="8"/>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A70" s="77"/>
+      <c r="A70" s="84"/>
       <c r="B70" s="42">
         <v>67</v>
       </c>
@@ -3237,11 +3242,11 @@
       <c r="F70" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G70" s="91"/>
+      <c r="G70" s="75"/>
       <c r="H70" s="8"/>
     </row>
     <row r="71" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A71" s="77"/>
+      <c r="A71" s="84"/>
       <c r="B71" s="42">
         <v>68</v>
       </c>
@@ -3255,10 +3260,10 @@
       <c r="F71" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G71" s="92"/>
+      <c r="G71" s="76"/>
     </row>
     <row r="72" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A72" s="77"/>
+      <c r="A72" s="84"/>
       <c r="B72" s="42">
         <v>69</v>
       </c>
@@ -3272,11 +3277,11 @@
       <c r="F72" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G72" s="91"/>
+      <c r="G72" s="75"/>
       <c r="H72" s="8"/>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A73" s="77"/>
+      <c r="A73" s="84"/>
       <c r="B73" s="42">
         <v>70</v>
       </c>
@@ -3290,11 +3295,11 @@
       <c r="F73" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G73" s="91"/>
+      <c r="G73" s="75"/>
       <c r="H73" s="8"/>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A74" s="77"/>
+      <c r="A74" s="84"/>
       <c r="B74" s="42">
         <v>71</v>
       </c>
@@ -3308,11 +3313,11 @@
       <c r="F74" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G74" s="91"/>
+      <c r="G74" s="75"/>
       <c r="H74" s="8"/>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A75" s="77"/>
+      <c r="A75" s="84"/>
       <c r="B75" s="42">
         <v>72</v>
       </c>
@@ -3326,11 +3331,11 @@
       <c r="F75" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G75" s="91"/>
+      <c r="G75" s="75"/>
       <c r="H75" s="8"/>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A76" s="77"/>
+      <c r="A76" s="84"/>
       <c r="B76" s="42">
         <v>73</v>
       </c>
@@ -3344,11 +3349,11 @@
       <c r="F76" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G76" s="91"/>
+      <c r="G76" s="75"/>
       <c r="H76" s="8"/>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A77" s="77"/>
+      <c r="A77" s="84"/>
       <c r="B77" s="42">
         <v>74</v>
       </c>
@@ -3362,11 +3367,11 @@
       <c r="F77" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G77" s="91"/>
+      <c r="G77" s="75"/>
       <c r="H77" s="8"/>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A78" s="77"/>
+      <c r="A78" s="84"/>
       <c r="B78" s="42">
         <v>75</v>
       </c>
@@ -3380,13 +3385,13 @@
       <c r="F78" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G78" s="91" t="s">
+      <c r="G78" s="75" t="s">
         <v>264</v>
       </c>
       <c r="H78" s="8"/>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A79" s="75" t="s">
+      <c r="A79" s="82" t="s">
         <v>96</v>
       </c>
       <c r="B79" s="43">
@@ -3400,13 +3405,13 @@
         <v>98</v>
       </c>
       <c r="F79" s="61" t="s">
-        <v>11</v>
-      </c>
-      <c r="G79" s="91"/>
+        <v>223</v>
+      </c>
+      <c r="G79" s="75"/>
       <c r="H79" s="8"/>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A80" s="75"/>
+      <c r="A80" s="82"/>
       <c r="B80" s="43">
         <v>77</v>
       </c>
@@ -3420,11 +3425,11 @@
       <c r="F80" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G80" s="91"/>
+      <c r="G80" s="75"/>
       <c r="H80" s="8"/>
     </row>
     <row r="81" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A81" s="75"/>
+      <c r="A81" s="82"/>
       <c r="B81" s="43">
         <v>78</v>
       </c>
@@ -3440,10 +3445,10 @@
       <c r="F81" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G81" s="95"/>
+      <c r="G81" s="79"/>
     </row>
     <row r="82" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A82" s="75"/>
+      <c r="A82" s="82"/>
       <c r="B82" s="43">
         <v>79</v>
       </c>
@@ -3457,10 +3462,10 @@
       <c r="F82" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G82" s="95"/>
+      <c r="G82" s="79"/>
     </row>
     <row r="83" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A83" s="75"/>
+      <c r="A83" s="82"/>
       <c r="B83" s="43">
         <v>80</v>
       </c>
@@ -3474,7 +3479,7 @@
       <c r="F83" s="61" t="s">
         <v>11</v>
       </c>
-      <c r="G83" s="92"/>
+      <c r="G83" s="76"/>
     </row>
     <row r="84" spans="1:7" x14ac:dyDescent="0.3">
       <c r="D84" s="4"/>
@@ -3612,26 +3617,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A1" s="86" t="s">
+      <c r="A1" s="93" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
-      <c r="D1" s="86"/>
-      <c r="E1" s="86"/>
-      <c r="F1" s="86"/>
-      <c r="G1" s="86"/>
+      <c r="B1" s="93"/>
+      <c r="C1" s="93"/>
+      <c r="D1" s="93"/>
+      <c r="E1" s="93"/>
+      <c r="F1" s="93"/>
+      <c r="G1" s="93"/>
     </row>
     <row r="2" spans="1:7" ht="28.5" x14ac:dyDescent="0.25">
-      <c r="A2" s="87" t="s">
+      <c r="A2" s="94" t="s">
         <v>104</v>
       </c>
-      <c r="B2" s="87"/>
-      <c r="C2" s="87"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="87"/>
+      <c r="B2" s="94"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="94"/>
+      <c r="E2" s="94"/>
+      <c r="F2" s="94"/>
+      <c r="G2" s="94"/>
     </row>
     <row r="3" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A3" s="35"/>
@@ -3649,7 +3654,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" s="21" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="84" t="s">
+      <c r="A4" s="91" t="s">
         <v>106</v>
       </c>
       <c r="B4" s="62">
@@ -3670,7 +3675,7 @@
       <c r="G4" s="20"/>
     </row>
     <row r="5" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A5" s="84"/>
+      <c r="A5" s="91"/>
       <c r="B5" s="62">
         <v>2</v>
       </c>
@@ -3687,7 +3692,7 @@
       <c r="G5" s="23"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A6" s="84"/>
+      <c r="A6" s="91"/>
       <c r="B6" s="62">
         <v>3</v>
       </c>
@@ -3704,7 +3709,7 @@
       <c r="G6" s="23"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A7" s="84"/>
+      <c r="A7" s="91"/>
       <c r="B7" s="62">
         <v>4</v>
       </c>
@@ -3721,7 +3726,7 @@
       <c r="G7" s="23"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" s="84"/>
+      <c r="A8" s="91"/>
       <c r="B8" s="62">
         <v>5</v>
       </c>
@@ -3738,7 +3743,7 @@
       <c r="G8" s="23"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="84"/>
+      <c r="A9" s="91"/>
       <c r="B9" s="62">
         <v>6</v>
       </c>
@@ -3755,7 +3760,7 @@
       <c r="G9" s="23"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="84"/>
+      <c r="A10" s="91"/>
       <c r="B10" s="62">
         <v>7</v>
       </c>
@@ -3772,7 +3777,7 @@
       <c r="G10" s="23"/>
     </row>
     <row r="11" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="88" t="s">
+      <c r="A11" s="95" t="s">
         <v>115</v>
       </c>
       <c r="B11" s="66">
@@ -3791,7 +3796,7 @@
       <c r="G11" s="23"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" s="88"/>
+      <c r="A12" s="95"/>
       <c r="B12" s="66">
         <v>9</v>
       </c>
@@ -3808,7 +3813,7 @@
       <c r="G12" s="23"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" s="88"/>
+      <c r="A13" s="95"/>
       <c r="B13" s="66">
         <v>10</v>
       </c>
@@ -3825,7 +3830,7 @@
       <c r="G13" s="23"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="88"/>
+      <c r="A14" s="95"/>
       <c r="B14" s="66">
         <v>11</v>
       </c>
@@ -3842,7 +3847,7 @@
       <c r="G14" s="36"/>
     </row>
     <row r="15" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A15" s="88"/>
+      <c r="A15" s="95"/>
       <c r="B15" s="66">
         <v>12</v>
       </c>
@@ -3859,7 +3864,7 @@
       <c r="G15" s="23"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="88"/>
+      <c r="A16" s="95"/>
       <c r="B16" s="66">
         <v>13</v>
       </c>
@@ -3876,7 +3881,7 @@
       <c r="G16" s="23"/>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A17" s="88"/>
+      <c r="A17" s="95"/>
       <c r="B17" s="66">
         <v>14</v>
       </c>
@@ -3893,7 +3898,7 @@
       <c r="G17" s="23"/>
     </row>
     <row r="18" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="88"/>
+      <c r="A18" s="95"/>
       <c r="B18" s="66">
         <v>15</v>
       </c>
@@ -3910,7 +3915,7 @@
       <c r="G18" s="23"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A19" s="88"/>
+      <c r="A19" s="95"/>
       <c r="B19" s="66">
         <v>16</v>
       </c>
@@ -3927,7 +3932,7 @@
       <c r="G19" s="23"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A20" s="88"/>
+      <c r="A20" s="95"/>
       <c r="B20" s="66">
         <v>17</v>
       </c>
@@ -3944,7 +3949,7 @@
       <c r="G20" s="23"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A21" s="88"/>
+      <c r="A21" s="95"/>
       <c r="B21" s="66">
         <v>18</v>
       </c>
@@ -3961,7 +3966,7 @@
       <c r="G21" s="23"/>
     </row>
     <row r="22" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="85" t="s">
+      <c r="A22" s="92" t="s">
         <v>128</v>
       </c>
       <c r="B22" s="72">
@@ -3980,7 +3985,7 @@
       <c r="G22" s="23"/>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="85"/>
+      <c r="A23" s="92"/>
       <c r="B23" s="72">
         <v>20</v>
       </c>
@@ -3997,7 +4002,7 @@
       <c r="G23" s="23"/>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A24" s="85"/>
+      <c r="A24" s="92"/>
       <c r="B24" s="72">
         <v>21</v>
       </c>
@@ -4014,7 +4019,7 @@
       <c r="G24" s="23"/>
     </row>
     <row r="25" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="85"/>
+      <c r="A25" s="92"/>
       <c r="B25" s="72">
         <v>22</v>
       </c>
@@ -4031,7 +4036,7 @@
       <c r="G25" s="23"/>
     </row>
     <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="85"/>
+      <c r="A26" s="92"/>
       <c r="B26" s="72">
         <v>23</v>
       </c>
@@ -4048,7 +4053,7 @@
       <c r="G26" s="23"/>
     </row>
     <row r="27" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A27" s="85"/>
+      <c r="A27" s="92"/>
       <c r="B27" s="72">
         <v>24</v>
       </c>
@@ -4065,7 +4070,7 @@
       <c r="G27" s="23"/>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A28" s="85"/>
+      <c r="A28" s="92"/>
       <c r="B28" s="72">
         <v>25</v>
       </c>
@@ -4082,7 +4087,7 @@
       <c r="G28" s="23"/>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A29" s="85"/>
+      <c r="A29" s="92"/>
       <c r="B29" s="72">
         <v>26</v>
       </c>
@@ -4099,7 +4104,7 @@
       <c r="G29" s="23"/>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A30" s="84" t="s">
+      <c r="A30" s="91" t="s">
         <v>137</v>
       </c>
       <c r="B30" s="62">
@@ -4118,7 +4123,7 @@
       <c r="G30" s="23"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A31" s="84"/>
+      <c r="A31" s="91"/>
       <c r="B31" s="62">
         <v>28</v>
       </c>
@@ -4135,7 +4140,7 @@
       <c r="G31" s="23"/>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A32" s="84"/>
+      <c r="A32" s="91"/>
       <c r="B32" s="62">
         <v>29</v>
       </c>
@@ -4152,7 +4157,7 @@
       <c r="G32" s="23"/>
     </row>
     <row r="33" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A33" s="84"/>
+      <c r="A33" s="91"/>
       <c r="B33" s="62">
         <v>30</v>
       </c>
@@ -4169,7 +4174,7 @@
       <c r="G33" s="23"/>
     </row>
     <row r="34" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A34" s="84"/>
+      <c r="A34" s="91"/>
       <c r="B34" s="62">
         <v>31</v>
       </c>
@@ -4186,7 +4191,7 @@
       <c r="G34" s="23"/>
     </row>
     <row r="35" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A35" s="84"/>
+      <c r="A35" s="91"/>
       <c r="B35" s="62">
         <v>32</v>
       </c>
@@ -4203,7 +4208,7 @@
       <c r="G35" s="23"/>
     </row>
     <row r="36" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A36" s="84"/>
+      <c r="A36" s="91"/>
       <c r="B36" s="62">
         <v>33</v>
       </c>
@@ -4220,7 +4225,7 @@
       <c r="G36" s="23"/>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A37" s="84"/>
+      <c r="A37" s="91"/>
       <c r="B37" s="62">
         <v>34</v>
       </c>
@@ -4237,7 +4242,7 @@
       <c r="G37" s="23"/>
     </row>
     <row r="38" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A38" s="84"/>
+      <c r="A38" s="91"/>
       <c r="B38" s="62">
         <v>35</v>
       </c>
@@ -4254,7 +4259,7 @@
       <c r="G38" s="23"/>
     </row>
     <row r="39" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A39" s="84"/>
+      <c r="A39" s="91"/>
       <c r="B39" s="62">
         <v>36</v>
       </c>
@@ -4271,7 +4276,7 @@
       <c r="G39" s="23"/>
     </row>
     <row r="40" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A40" s="84"/>
+      <c r="A40" s="91"/>
       <c r="B40" s="62">
         <v>37</v>
       </c>
@@ -4288,7 +4293,7 @@
       <c r="G40" s="23"/>
     </row>
     <row r="41" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A41" s="84"/>
+      <c r="A41" s="91"/>
       <c r="B41" s="62">
         <v>38</v>
       </c>
@@ -4305,7 +4310,7 @@
       <c r="G41" s="23"/>
     </row>
     <row r="42" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A42" s="84"/>
+      <c r="A42" s="91"/>
       <c r="B42" s="62">
         <v>39</v>
       </c>
@@ -4322,7 +4327,7 @@
       <c r="G42" s="23"/>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A43" s="84"/>
+      <c r="A43" s="91"/>
       <c r="B43" s="62">
         <v>40</v>
       </c>
@@ -4339,7 +4344,7 @@
       <c r="G43" s="23"/>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A44" s="84"/>
+      <c r="A44" s="91"/>
       <c r="B44" s="62">
         <v>41</v>
       </c>
@@ -4356,7 +4361,7 @@
       <c r="G44" s="23"/>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A45" s="84"/>
+      <c r="A45" s="91"/>
       <c r="B45" s="62">
         <v>42</v>
       </c>
@@ -4373,7 +4378,7 @@
       <c r="G45" s="23"/>
     </row>
     <row r="46" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A46" s="84"/>
+      <c r="A46" s="91"/>
       <c r="B46" s="62">
         <v>43</v>
       </c>
@@ -4390,7 +4395,7 @@
       <c r="G46" s="23"/>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A47" s="88" t="s">
+      <c r="A47" s="95" t="s">
         <v>157</v>
       </c>
       <c r="B47" s="66">
@@ -4409,7 +4414,7 @@
       <c r="G47" s="23"/>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A48" s="88"/>
+      <c r="A48" s="95"/>
       <c r="B48" s="66">
         <v>45</v>
       </c>
@@ -4426,7 +4431,7 @@
       <c r="G48" s="23"/>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A49" s="88"/>
+      <c r="A49" s="95"/>
       <c r="B49" s="66">
         <v>46</v>
       </c>
@@ -4443,7 +4448,7 @@
       <c r="G49" s="23"/>
     </row>
     <row r="50" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A50" s="88"/>
+      <c r="A50" s="95"/>
       <c r="B50" s="66">
         <v>47</v>
       </c>
@@ -4460,7 +4465,7 @@
       <c r="G50" s="23"/>
     </row>
     <row r="51" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A51" s="88"/>
+      <c r="A51" s="95"/>
       <c r="B51" s="66">
         <v>48</v>
       </c>
@@ -4477,7 +4482,7 @@
       <c r="G51" s="23"/>
     </row>
     <row r="52" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A52" s="88"/>
+      <c r="A52" s="95"/>
       <c r="B52" s="66">
         <v>49</v>
       </c>
@@ -4494,7 +4499,7 @@
       <c r="G52" s="23"/>
     </row>
     <row r="53" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A53" s="88"/>
+      <c r="A53" s="95"/>
       <c r="B53" s="66">
         <v>50</v>
       </c>
@@ -4511,7 +4516,7 @@
       <c r="G53" s="23"/>
     </row>
     <row r="54" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A54" s="88"/>
+      <c r="A54" s="95"/>
       <c r="B54" s="66">
         <v>51</v>
       </c>
@@ -4528,7 +4533,7 @@
       <c r="G54" s="23"/>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A55" s="88"/>
+      <c r="A55" s="95"/>
       <c r="B55" s="66">
         <v>52</v>
       </c>
@@ -4545,7 +4550,7 @@
       <c r="G55" s="23"/>
     </row>
     <row r="56" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A56" s="88"/>
+      <c r="A56" s="95"/>
       <c r="B56" s="66">
         <v>53</v>
       </c>
@@ -4562,7 +4567,7 @@
       <c r="G56" s="23"/>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="88"/>
+      <c r="A57" s="95"/>
       <c r="B57" s="66">
         <v>54</v>
       </c>
@@ -4579,7 +4584,7 @@
       <c r="G57" s="23"/>
     </row>
     <row r="58" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A58" s="88"/>
+      <c r="A58" s="95"/>
       <c r="B58" s="66">
         <v>55</v>
       </c>
@@ -4596,7 +4601,7 @@
       <c r="G58" s="23"/>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A59" s="88"/>
+      <c r="A59" s="95"/>
       <c r="B59" s="66">
         <v>56</v>
       </c>
@@ -4613,7 +4618,7 @@
       <c r="G59" s="23"/>
     </row>
     <row r="60" spans="1:7" ht="75" x14ac:dyDescent="0.25">
-      <c r="A60" s="88"/>
+      <c r="A60" s="95"/>
       <c r="B60" s="66">
         <v>57</v>
       </c>
@@ -4630,7 +4635,7 @@
       <c r="G60" s="23"/>
     </row>
     <row r="61" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A61" s="88"/>
+      <c r="A61" s="95"/>
       <c r="B61" s="66">
         <v>58</v>
       </c>
@@ -4647,7 +4652,7 @@
       <c r="G61" s="23"/>
     </row>
     <row r="62" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A62" s="88"/>
+      <c r="A62" s="95"/>
       <c r="B62" s="66">
         <v>59</v>
       </c>
@@ -4664,7 +4669,7 @@
       <c r="G62" s="23"/>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="88"/>
+      <c r="A63" s="95"/>
       <c r="B63" s="66">
         <v>60</v>
       </c>
@@ -4681,7 +4686,7 @@
       <c r="G63" s="23"/>
     </row>
     <row r="64" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A64" s="88"/>
+      <c r="A64" s="95"/>
       <c r="B64" s="66">
         <v>61</v>
       </c>
@@ -4698,7 +4703,7 @@
       <c r="G64" s="23"/>
     </row>
     <row r="65" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A65" s="88"/>
+      <c r="A65" s="95"/>
       <c r="B65" s="66">
         <v>62</v>
       </c>
@@ -4715,7 +4720,7 @@
       <c r="G65" s="23"/>
     </row>
     <row r="66" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A66" s="88"/>
+      <c r="A66" s="95"/>
       <c r="B66" s="66">
         <v>63</v>
       </c>
@@ -4732,7 +4737,7 @@
       <c r="G66" s="23"/>
     </row>
     <row r="67" spans="1:7" ht="30" x14ac:dyDescent="0.25">
-      <c r="A67" s="88"/>
+      <c r="A67" s="95"/>
       <c r="B67" s="66">
         <v>64</v>
       </c>
@@ -4749,7 +4754,7 @@
       <c r="G67" s="23"/>
     </row>
     <row r="68" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A68" s="88"/>
+      <c r="A68" s="95"/>
       <c r="B68" s="66">
         <v>65</v>
       </c>
@@ -4766,7 +4771,7 @@
       <c r="G68" s="23"/>
     </row>
     <row r="69" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A69" s="88"/>
+      <c r="A69" s="95"/>
       <c r="B69" s="66">
         <v>66</v>
       </c>
@@ -4783,7 +4788,7 @@
       <c r="G69" s="23"/>
     </row>
     <row r="70" spans="1:7" ht="60" x14ac:dyDescent="0.25">
-      <c r="A70" s="88"/>
+      <c r="A70" s="95"/>
       <c r="B70" s="66">
         <v>67</v>
       </c>
@@ -4800,7 +4805,7 @@
       <c r="G70" s="23"/>
     </row>
     <row r="71" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A71" s="85" t="s">
+      <c r="A71" s="92" t="s">
         <v>189</v>
       </c>
       <c r="B71" s="72">
@@ -4819,7 +4824,7 @@
       <c r="G71" s="23"/>
     </row>
     <row r="72" spans="1:7" ht="45" x14ac:dyDescent="0.25">
-      <c r="A72" s="85"/>
+      <c r="A72" s="92"/>
       <c r="B72" s="72">
         <v>69</v>
       </c>
@@ -4836,7 +4841,7 @@
       <c r="G72" s="23"/>
     </row>
     <row r="73" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A73" s="85"/>
+      <c r="A73" s="92"/>
       <c r="B73" s="72">
         <v>70</v>
       </c>
@@ -4853,7 +4858,7 @@
       <c r="G73" s="23"/>
     </row>
     <row r="74" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A74" s="85"/>
+      <c r="A74" s="92"/>
       <c r="B74" s="72">
         <v>71</v>
       </c>
@@ -4870,7 +4875,7 @@
       <c r="G74" s="23"/>
     </row>
     <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A75" s="85"/>
+      <c r="A75" s="92"/>
       <c r="B75" s="72">
         <v>72</v>
       </c>
@@ -4887,7 +4892,7 @@
       <c r="G75" s="23"/>
     </row>
     <row r="76" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A76" s="83" t="s">
+      <c r="A76" s="90" t="s">
         <v>196</v>
       </c>
       <c r="B76" s="62">
@@ -4906,7 +4911,7 @@
       <c r="G76" s="23"/>
     </row>
     <row r="77" spans="1:7" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="84"/>
+      <c r="A77" s="91"/>
       <c r="B77" s="62">
         <v>74</v>
       </c>
@@ -5046,20 +5051,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A1" s="89" t="s">
+      <c r="A1" s="96" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="89"/>
-      <c r="C1" s="89"/>
-      <c r="D1" s="89"/>
+      <c r="B1" s="96"/>
+      <c r="C1" s="96"/>
+      <c r="D1" s="96"/>
     </row>
     <row r="2" spans="1:4" ht="28.5" x14ac:dyDescent="0.45">
-      <c r="A2" s="90" t="s">
+      <c r="A2" s="97" t="s">
         <v>199</v>
       </c>
-      <c r="B2" s="90"/>
-      <c r="C2" s="90"/>
-      <c r="D2" s="90"/>
+      <c r="B2" s="97"/>
+      <c r="C2" s="97"/>
+      <c r="D2" s="97"/>
     </row>
     <row r="3" spans="1:4" ht="21" x14ac:dyDescent="0.35">
       <c r="A3" s="26"/>

</xml_diff>